<commit_message>
Mise à jour Garde — 23/04/2026
</commit_message>
<xml_diff>
--- a/data/export_garde.xlsx
+++ b/data/export_garde.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="369">
   <si>
     <t>Début</t>
   </si>
@@ -1091,6 +1091,27 @@
   </si>
   <si>
     <t>22-04-2026</t>
+  </si>
+  <si>
+    <t>25-04-2026</t>
+  </si>
+  <si>
+    <t>[PROV] BSPP</t>
+  </si>
+  <si>
+    <t>30-04-2026</t>
+  </si>
+  <si>
+    <t>04-05-2026</t>
+  </si>
+  <si>
+    <t>16-05-2026</t>
+  </si>
+  <si>
+    <t>BSPP - Journée des CS</t>
+  </si>
+  <si>
+    <t>TBC</t>
   </si>
   <si>
     <t>14-06-2026</t>
@@ -1459,7 +1480,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:N341"/>
+  <dimension ref="A1:N345"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854004" bestFit="true" customWidth="true" style="0"/>
@@ -13171,12 +13192,24 @@
       <c r="D337" t="s">
         <v>112</v>
       </c>
-      <c r="E337"/>
-      <c r="F337"/>
-      <c r="G337"/>
-      <c r="H337"/>
-      <c r="I337"/>
-      <c r="J337"/>
+      <c r="E337">
+        <v>4</v>
+      </c>
+      <c r="F337">
+        <v>4</v>
+      </c>
+      <c r="G337">
+        <v>0</v>
+      </c>
+      <c r="H337">
+        <v>0</v>
+      </c>
+      <c r="I337">
+        <v>4</v>
+      </c>
+      <c r="J337">
+        <v>0</v>
+      </c>
       <c r="K337">
         <v>10</v>
       </c>
@@ -13199,11 +13232,17 @@
       <c r="D338" t="s">
         <v>16</v>
       </c>
-      <c r="E338"/>
-      <c r="F338"/>
+      <c r="E338">
+        <v>3</v>
+      </c>
+      <c r="F338">
+        <v>2</v>
+      </c>
       <c r="G338"/>
       <c r="H338"/>
-      <c r="I338"/>
+      <c r="I338">
+        <v>3</v>
+      </c>
       <c r="J338"/>
       <c r="K338">
         <v>6</v>
@@ -13227,12 +13266,24 @@
       <c r="D339" t="s">
         <v>108</v>
       </c>
-      <c r="E339"/>
-      <c r="F339"/>
-      <c r="G339"/>
-      <c r="H339"/>
-      <c r="I339"/>
-      <c r="J339"/>
+      <c r="E339">
+        <v>3</v>
+      </c>
+      <c r="F339">
+        <v>3</v>
+      </c>
+      <c r="G339">
+        <v>0</v>
+      </c>
+      <c r="H339">
+        <v>0</v>
+      </c>
+      <c r="I339">
+        <v>3</v>
+      </c>
+      <c r="J339">
+        <v>0</v>
+      </c>
       <c r="K339">
         <v>6</v>
       </c>
@@ -13253,7 +13304,7 @@
       </c>
       <c r="C340"/>
       <c r="D340" t="s">
-        <v>28</v>
+        <v>283</v>
       </c>
       <c r="E340"/>
       <c r="F340"/>
@@ -13262,13 +13313,13 @@
       <c r="I340"/>
       <c r="J340"/>
       <c r="K340">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L340">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M340">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N340"/>
     </row>
@@ -13277,11 +13328,11 @@
         <v>360</v>
       </c>
       <c r="B341" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C341"/>
       <c r="D341" t="s">
-        <v>20</v>
+        <v>167</v>
       </c>
       <c r="E341"/>
       <c r="F341"/>
@@ -13290,15 +13341,127 @@
       <c r="I341"/>
       <c r="J341"/>
       <c r="K341">
+        <v>6</v>
+      </c>
+      <c r="L341">
+        <v>4</v>
+      </c>
+      <c r="M341">
+        <v>24</v>
+      </c>
+      <c r="N341"/>
+    </row>
+    <row r="342" spans="1:14">
+      <c r="A342" t="s">
+        <v>361</v>
+      </c>
+      <c r="B342" t="s">
+        <v>359</v>
+      </c>
+      <c r="C342"/>
+      <c r="D342" t="s">
+        <v>335</v>
+      </c>
+      <c r="E342"/>
+      <c r="F342"/>
+      <c r="G342"/>
+      <c r="H342"/>
+      <c r="I342"/>
+      <c r="J342"/>
+      <c r="K342">
+        <v>6</v>
+      </c>
+      <c r="L342">
+        <v>2</v>
+      </c>
+      <c r="M342">
+        <v>12</v>
+      </c>
+      <c r="N342"/>
+    </row>
+    <row r="343" spans="1:14">
+      <c r="A343" t="s">
+        <v>362</v>
+      </c>
+      <c r="B343" t="s">
+        <v>363</v>
+      </c>
+      <c r="C343"/>
+      <c r="D343" t="s">
+        <v>364</v>
+      </c>
+      <c r="E343"/>
+      <c r="F343"/>
+      <c r="G343"/>
+      <c r="H343"/>
+      <c r="I343"/>
+      <c r="J343"/>
+      <c r="K343">
+        <v>8</v>
+      </c>
+      <c r="L343">
+        <v>1</v>
+      </c>
+      <c r="M343">
+        <v>8</v>
+      </c>
+      <c r="N343"/>
+    </row>
+    <row r="344" spans="1:14">
+      <c r="A344" t="s">
+        <v>365</v>
+      </c>
+      <c r="B344" t="s">
+        <v>366</v>
+      </c>
+      <c r="C344"/>
+      <c r="D344" t="s">
+        <v>28</v>
+      </c>
+      <c r="E344"/>
+      <c r="F344"/>
+      <c r="G344"/>
+      <c r="H344"/>
+      <c r="I344"/>
+      <c r="J344"/>
+      <c r="K344">
         <v>10</v>
       </c>
-      <c r="L341">
-        <v>4</v>
-      </c>
-      <c r="M341">
+      <c r="L344">
+        <v>1</v>
+      </c>
+      <c r="M344">
+        <v>10</v>
+      </c>
+      <c r="N344"/>
+    </row>
+    <row r="345" spans="1:14">
+      <c r="A345" t="s">
+        <v>367</v>
+      </c>
+      <c r="B345" t="s">
+        <v>368</v>
+      </c>
+      <c r="C345"/>
+      <c r="D345" t="s">
+        <v>20</v>
+      </c>
+      <c r="E345"/>
+      <c r="F345"/>
+      <c r="G345"/>
+      <c r="H345"/>
+      <c r="I345"/>
+      <c r="J345"/>
+      <c r="K345">
+        <v>10</v>
+      </c>
+      <c r="L345">
+        <v>4</v>
+      </c>
+      <c r="M345">
         <v>40</v>
       </c>
-      <c r="N341"/>
+      <c r="N345"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
Mise à jour Garde — 04/05/2026
</commit_message>
<xml_diff>
--- a/data/export_garde.xlsx
+++ b/data/export_garde.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="375">
   <si>
     <t>Début</t>
   </si>
@@ -1096,15 +1096,21 @@
     <t>25-04-2026</t>
   </si>
   <si>
+    <t>29-04-2026</t>
+  </si>
+  <si>
+    <t>30-04-2026</t>
+  </si>
+  <si>
+    <t>04-05-2026</t>
+  </si>
+  <si>
+    <t>11-05-2026</t>
+  </si>
+  <si>
     <t>[PROV] BSPP</t>
   </si>
   <si>
-    <t>30-04-2026</t>
-  </si>
-  <si>
-    <t>04-05-2026</t>
-  </si>
-  <si>
     <t>16-05-2026</t>
   </si>
   <si>
@@ -1112,6 +1118,18 @@
   </si>
   <si>
     <t>TBC</t>
+  </si>
+  <si>
+    <t>29-05-2026</t>
+  </si>
+  <si>
+    <t>[PROV] Garde BSPP</t>
+  </si>
+  <si>
+    <t>06-06-2026</t>
+  </si>
+  <si>
+    <t>08-06-2026</t>
   </si>
   <si>
     <t>14-06-2026</t>
@@ -1480,7 +1498,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:N345"/>
+  <dimension ref="A1:N352"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854004" bestFit="true" customWidth="true" style="0"/>
@@ -13300,14 +13318,18 @@
         <v>358</v>
       </c>
       <c r="B340" t="s">
-        <v>359</v>
+        <v>15</v>
       </c>
       <c r="C340"/>
       <c r="D340" t="s">
         <v>283</v>
       </c>
-      <c r="E340"/>
-      <c r="F340"/>
+      <c r="E340">
+        <v>4</v>
+      </c>
+      <c r="F340">
+        <v>4</v>
+      </c>
       <c r="G340"/>
       <c r="H340"/>
       <c r="I340"/>
@@ -13316,79 +13338,99 @@
         <v>6</v>
       </c>
       <c r="L340">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M340">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="N340"/>
     </row>
     <row r="341" spans="1:14">
       <c r="A341" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B341" t="s">
-        <v>359</v>
+        <v>15</v>
       </c>
       <c r="C341"/>
       <c r="D341" t="s">
-        <v>167</v>
-      </c>
-      <c r="E341"/>
-      <c r="F341"/>
-      <c r="G341"/>
-      <c r="H341"/>
-      <c r="I341"/>
-      <c r="J341"/>
+        <v>192</v>
+      </c>
+      <c r="E341">
+        <v>4</v>
+      </c>
+      <c r="F341">
+        <v>2</v>
+      </c>
+      <c r="G341">
+        <v>0</v>
+      </c>
+      <c r="H341">
+        <v>0</v>
+      </c>
+      <c r="I341">
+        <v>4</v>
+      </c>
+      <c r="J341">
+        <v>1</v>
+      </c>
       <c r="K341">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="L341">
         <v>4</v>
       </c>
       <c r="M341">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="N341"/>
     </row>
     <row r="342" spans="1:14">
       <c r="A342" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B342" t="s">
-        <v>359</v>
+        <v>15</v>
       </c>
       <c r="C342"/>
       <c r="D342" t="s">
-        <v>335</v>
-      </c>
-      <c r="E342"/>
-      <c r="F342"/>
+        <v>167</v>
+      </c>
+      <c r="E342">
+        <v>4</v>
+      </c>
+      <c r="F342">
+        <v>2</v>
+      </c>
       <c r="G342"/>
       <c r="H342"/>
-      <c r="I342"/>
-      <c r="J342"/>
+      <c r="I342">
+        <v>4</v>
+      </c>
+      <c r="J342">
+        <v>1</v>
+      </c>
       <c r="K342">
         <v>6</v>
       </c>
       <c r="L342">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M342">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="N342"/>
     </row>
     <row r="343" spans="1:14">
       <c r="A343" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B343" t="s">
-        <v>363</v>
+        <v>15</v>
       </c>
       <c r="C343"/>
       <c r="D343" t="s">
-        <v>364</v>
+        <v>335</v>
       </c>
       <c r="E343"/>
       <c r="F343"/>
@@ -13397,26 +13439,26 @@
       <c r="I343"/>
       <c r="J343"/>
       <c r="K343">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L343">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M343">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="N343"/>
     </row>
     <row r="344" spans="1:14">
       <c r="A344" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B344" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="C344"/>
       <c r="D344" t="s">
-        <v>28</v>
+        <v>230</v>
       </c>
       <c r="E344"/>
       <c r="F344"/>
@@ -13425,26 +13467,26 @@
       <c r="I344"/>
       <c r="J344"/>
       <c r="K344">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L344">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M344">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="N344"/>
     </row>
     <row r="345" spans="1:14">
       <c r="A345" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="B345" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="C345"/>
       <c r="D345" t="s">
-        <v>20</v>
+        <v>167</v>
       </c>
       <c r="E345"/>
       <c r="F345"/>
@@ -13453,15 +13495,211 @@
       <c r="I345"/>
       <c r="J345"/>
       <c r="K345">
+        <v>6</v>
+      </c>
+      <c r="L345">
+        <v>1</v>
+      </c>
+      <c r="M345">
+        <v>6</v>
+      </c>
+      <c r="N345"/>
+    </row>
+    <row r="346" spans="1:14">
+      <c r="A346" t="s">
+        <v>364</v>
+      </c>
+      <c r="B346" t="s">
+        <v>365</v>
+      </c>
+      <c r="C346"/>
+      <c r="D346" t="s">
+        <v>366</v>
+      </c>
+      <c r="E346"/>
+      <c r="F346"/>
+      <c r="G346"/>
+      <c r="H346"/>
+      <c r="I346"/>
+      <c r="J346"/>
+      <c r="K346">
+        <v>8</v>
+      </c>
+      <c r="L346">
+        <v>3</v>
+      </c>
+      <c r="M346">
+        <v>24</v>
+      </c>
+      <c r="N346"/>
+    </row>
+    <row r="347" spans="1:14">
+      <c r="A347" t="s">
+        <v>364</v>
+      </c>
+      <c r="B347" t="s">
+        <v>363</v>
+      </c>
+      <c r="C347"/>
+      <c r="D347" t="s">
+        <v>136</v>
+      </c>
+      <c r="E347"/>
+      <c r="F347"/>
+      <c r="G347"/>
+      <c r="H347"/>
+      <c r="I347"/>
+      <c r="J347"/>
+      <c r="K347">
+        <v>9</v>
+      </c>
+      <c r="L347">
+        <v>1</v>
+      </c>
+      <c r="M347">
+        <v>9</v>
+      </c>
+      <c r="N347"/>
+    </row>
+    <row r="348" spans="1:14">
+      <c r="A348" t="s">
+        <v>367</v>
+      </c>
+      <c r="B348" t="s">
+        <v>368</v>
+      </c>
+      <c r="C348"/>
+      <c r="D348" t="s">
+        <v>103</v>
+      </c>
+      <c r="E348"/>
+      <c r="F348"/>
+      <c r="G348"/>
+      <c r="H348"/>
+      <c r="I348"/>
+      <c r="J348"/>
+      <c r="K348">
+        <v>12</v>
+      </c>
+      <c r="L348">
+        <v>2</v>
+      </c>
+      <c r="M348">
+        <v>24</v>
+      </c>
+      <c r="N348"/>
+    </row>
+    <row r="349" spans="1:14">
+      <c r="A349" t="s">
+        <v>369</v>
+      </c>
+      <c r="B349" t="s">
+        <v>368</v>
+      </c>
+      <c r="C349"/>
+      <c r="D349" t="s">
+        <v>192</v>
+      </c>
+      <c r="E349"/>
+      <c r="F349"/>
+      <c r="G349"/>
+      <c r="H349"/>
+      <c r="I349"/>
+      <c r="J349"/>
+      <c r="K349">
+        <v>12</v>
+      </c>
+      <c r="L349">
+        <v>3</v>
+      </c>
+      <c r="M349">
+        <v>36</v>
+      </c>
+      <c r="N349"/>
+    </row>
+    <row r="350" spans="1:14">
+      <c r="A350" t="s">
+        <v>370</v>
+      </c>
+      <c r="B350" t="s">
+        <v>368</v>
+      </c>
+      <c r="C350"/>
+      <c r="D350" t="s">
+        <v>16</v>
+      </c>
+      <c r="E350"/>
+      <c r="F350"/>
+      <c r="G350"/>
+      <c r="H350"/>
+      <c r="I350"/>
+      <c r="J350"/>
+      <c r="K350">
+        <v>6</v>
+      </c>
+      <c r="L350">
+        <v>2</v>
+      </c>
+      <c r="M350">
+        <v>12</v>
+      </c>
+      <c r="N350"/>
+    </row>
+    <row r="351" spans="1:14">
+      <c r="A351" t="s">
+        <v>371</v>
+      </c>
+      <c r="B351" t="s">
+        <v>372</v>
+      </c>
+      <c r="C351"/>
+      <c r="D351" t="s">
+        <v>28</v>
+      </c>
+      <c r="E351"/>
+      <c r="F351"/>
+      <c r="G351"/>
+      <c r="H351"/>
+      <c r="I351"/>
+      <c r="J351"/>
+      <c r="K351">
         <v>10</v>
       </c>
-      <c r="L345">
-        <v>4</v>
-      </c>
-      <c r="M345">
+      <c r="L351">
+        <v>1</v>
+      </c>
+      <c r="M351">
+        <v>10</v>
+      </c>
+      <c r="N351"/>
+    </row>
+    <row r="352" spans="1:14">
+      <c r="A352" t="s">
+        <v>373</v>
+      </c>
+      <c r="B352" t="s">
+        <v>374</v>
+      </c>
+      <c r="C352"/>
+      <c r="D352" t="s">
+        <v>20</v>
+      </c>
+      <c r="E352"/>
+      <c r="F352"/>
+      <c r="G352"/>
+      <c r="H352"/>
+      <c r="I352"/>
+      <c r="J352"/>
+      <c r="K352">
+        <v>10</v>
+      </c>
+      <c r="L352">
+        <v>4</v>
+      </c>
+      <c r="M352">
         <v>40</v>
       </c>
-      <c r="N345"/>
+      <c r="N352"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
Mise à jour Garde — 13/05/2026
</commit_message>
<xml_diff>
--- a/data/export_garde.xlsx
+++ b/data/export_garde.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="380">
   <si>
     <t>Début</t>
   </si>
@@ -1108,7 +1108,10 @@
     <t>11-05-2026</t>
   </si>
   <si>
-    <t>[PROV] BSPP</t>
+    <t>13-05-2026</t>
+  </si>
+  <si>
+    <t>14-05-2026</t>
   </si>
   <si>
     <t>16-05-2026</t>
@@ -1117,7 +1120,13 @@
     <t>BSPP - Journée des CS</t>
   </si>
   <si>
-    <t>TBC</t>
+    <t>CHTO</t>
+  </si>
+  <si>
+    <t>19-05-2026</t>
+  </si>
+  <si>
+    <t>23-05-2026</t>
   </si>
   <si>
     <t>29-05-2026</t>
@@ -1130,6 +1139,12 @@
   </si>
   <si>
     <t>08-06-2026</t>
+  </si>
+  <si>
+    <t>09-06-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[PROV] Garde BSPP </t>
   </si>
   <si>
     <t>14-06-2026</t>
@@ -1498,7 +1513,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:N352"/>
+  <dimension ref="A1:N358"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854004" bestFit="true" customWidth="true" style="0"/>
@@ -13432,12 +13447,24 @@
       <c r="D343" t="s">
         <v>335</v>
       </c>
-      <c r="E343"/>
-      <c r="F343"/>
-      <c r="G343"/>
-      <c r="H343"/>
-      <c r="I343"/>
-      <c r="J343"/>
+      <c r="E343">
+        <v>3</v>
+      </c>
+      <c r="F343">
+        <v>3</v>
+      </c>
+      <c r="G343">
+        <v>0</v>
+      </c>
+      <c r="H343">
+        <v>0</v>
+      </c>
+      <c r="I343">
+        <v>3</v>
+      </c>
+      <c r="J343">
+        <v>0</v>
+      </c>
       <c r="K343">
         <v>6</v>
       </c>
@@ -13454,26 +13481,38 @@
         <v>362</v>
       </c>
       <c r="B344" t="s">
-        <v>363</v>
+        <v>232</v>
       </c>
       <c r="C344"/>
       <c r="D344" t="s">
         <v>230</v>
       </c>
-      <c r="E344"/>
-      <c r="F344"/>
-      <c r="G344"/>
-      <c r="H344"/>
-      <c r="I344"/>
-      <c r="J344"/>
+      <c r="E344">
+        <v>3</v>
+      </c>
+      <c r="F344">
+        <v>3</v>
+      </c>
+      <c r="G344">
+        <v>0</v>
+      </c>
+      <c r="H344">
+        <v>0</v>
+      </c>
+      <c r="I344">
+        <v>3</v>
+      </c>
+      <c r="J344">
+        <v>0</v>
+      </c>
       <c r="K344">
         <v>6</v>
       </c>
       <c r="L344">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M344">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="N344"/>
     </row>
@@ -13482,39 +13521,51 @@
         <v>362</v>
       </c>
       <c r="B345" t="s">
-        <v>363</v>
+        <v>15</v>
       </c>
       <c r="C345"/>
       <c r="D345" t="s">
         <v>167</v>
       </c>
-      <c r="E345"/>
-      <c r="F345"/>
-      <c r="G345"/>
-      <c r="H345"/>
-      <c r="I345"/>
-      <c r="J345"/>
+      <c r="E345">
+        <v>3</v>
+      </c>
+      <c r="F345">
+        <v>3</v>
+      </c>
+      <c r="G345">
+        <v>0</v>
+      </c>
+      <c r="H345">
+        <v>0</v>
+      </c>
+      <c r="I345">
+        <v>4</v>
+      </c>
+      <c r="J345">
+        <v>0</v>
+      </c>
       <c r="K345">
         <v>6</v>
       </c>
       <c r="L345">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M345">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="N345"/>
     </row>
     <row r="346" spans="1:14">
       <c r="A346" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B346" t="s">
-        <v>365</v>
+        <v>227</v>
       </c>
       <c r="C346"/>
       <c r="D346" t="s">
-        <v>366</v>
+        <v>256</v>
       </c>
       <c r="E346"/>
       <c r="F346"/>
@@ -13523,10 +13574,10 @@
       <c r="I346"/>
       <c r="J346"/>
       <c r="K346">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L346">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M346">
         <v>24</v>
@@ -13538,11 +13589,11 @@
         <v>364</v>
       </c>
       <c r="B347" t="s">
-        <v>363</v>
+        <v>15</v>
       </c>
       <c r="C347"/>
       <c r="D347" t="s">
-        <v>136</v>
+        <v>256</v>
       </c>
       <c r="E347"/>
       <c r="F347"/>
@@ -13551,26 +13602,26 @@
       <c r="I347"/>
       <c r="J347"/>
       <c r="K347">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L347">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M347">
-        <v>9</v>
+        <v>60</v>
       </c>
       <c r="N347"/>
     </row>
     <row r="348" spans="1:14">
       <c r="A348" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B348" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C348"/>
       <c r="D348" t="s">
-        <v>103</v>
+        <v>367</v>
       </c>
       <c r="E348"/>
       <c r="F348"/>
@@ -13579,26 +13630,26 @@
       <c r="I348"/>
       <c r="J348"/>
       <c r="K348">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="L348">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M348">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="N348"/>
     </row>
     <row r="349" spans="1:14">
       <c r="A349" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="B349" t="s">
-        <v>368</v>
+        <v>15</v>
       </c>
       <c r="C349"/>
       <c r="D349" t="s">
-        <v>192</v>
+        <v>136</v>
       </c>
       <c r="E349"/>
       <c r="F349"/>
@@ -13619,14 +13670,14 @@
     </row>
     <row r="350" spans="1:14">
       <c r="A350" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B350" t="s">
-        <v>368</v>
+        <v>227</v>
       </c>
       <c r="C350"/>
       <c r="D350" t="s">
-        <v>16</v>
+        <v>257</v>
       </c>
       <c r="E350"/>
       <c r="F350"/>
@@ -13635,26 +13686,26 @@
       <c r="I350"/>
       <c r="J350"/>
       <c r="K350">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L350">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M350">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="N350"/>
     </row>
     <row r="351" spans="1:14">
       <c r="A351" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B351" t="s">
-        <v>372</v>
+        <v>227</v>
       </c>
       <c r="C351"/>
       <c r="D351" t="s">
-        <v>28</v>
+        <v>230</v>
       </c>
       <c r="E351"/>
       <c r="F351"/>
@@ -13663,26 +13714,26 @@
       <c r="I351"/>
       <c r="J351"/>
       <c r="K351">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L351">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M351">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="N351"/>
     </row>
     <row r="352" spans="1:14">
       <c r="A352" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="B352" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="C352"/>
       <c r="D352" t="s">
-        <v>20</v>
+        <v>103</v>
       </c>
       <c r="E352"/>
       <c r="F352"/>
@@ -13691,15 +13742,183 @@
       <c r="I352"/>
       <c r="J352"/>
       <c r="K352">
+        <v>12</v>
+      </c>
+      <c r="L352">
+        <v>4</v>
+      </c>
+      <c r="M352">
+        <v>48</v>
+      </c>
+      <c r="N352"/>
+    </row>
+    <row r="353" spans="1:14">
+      <c r="A353" t="s">
+        <v>370</v>
+      </c>
+      <c r="B353" t="s">
+        <v>371</v>
+      </c>
+      <c r="C353"/>
+      <c r="D353" t="s">
+        <v>256</v>
+      </c>
+      <c r="E353"/>
+      <c r="F353"/>
+      <c r="G353"/>
+      <c r="H353"/>
+      <c r="I353"/>
+      <c r="J353"/>
+      <c r="K353">
+        <v>6</v>
+      </c>
+      <c r="L353">
+        <v>6</v>
+      </c>
+      <c r="M353">
+        <v>36</v>
+      </c>
+      <c r="N353"/>
+    </row>
+    <row r="354" spans="1:14">
+      <c r="A354" t="s">
+        <v>372</v>
+      </c>
+      <c r="B354" t="s">
+        <v>371</v>
+      </c>
+      <c r="C354"/>
+      <c r="D354" t="s">
+        <v>192</v>
+      </c>
+      <c r="E354"/>
+      <c r="F354"/>
+      <c r="G354"/>
+      <c r="H354"/>
+      <c r="I354"/>
+      <c r="J354"/>
+      <c r="K354">
+        <v>12</v>
+      </c>
+      <c r="L354">
+        <v>5</v>
+      </c>
+      <c r="M354">
+        <v>60</v>
+      </c>
+      <c r="N354"/>
+    </row>
+    <row r="355" spans="1:14">
+      <c r="A355" t="s">
+        <v>373</v>
+      </c>
+      <c r="B355" t="s">
+        <v>371</v>
+      </c>
+      <c r="C355"/>
+      <c r="D355" t="s">
+        <v>16</v>
+      </c>
+      <c r="E355"/>
+      <c r="F355"/>
+      <c r="G355"/>
+      <c r="H355"/>
+      <c r="I355"/>
+      <c r="J355"/>
+      <c r="K355">
+        <v>6</v>
+      </c>
+      <c r="L355">
+        <v>5</v>
+      </c>
+      <c r="M355">
+        <v>30</v>
+      </c>
+      <c r="N355"/>
+    </row>
+    <row r="356" spans="1:14">
+      <c r="A356" t="s">
+        <v>374</v>
+      </c>
+      <c r="B356" t="s">
+        <v>375</v>
+      </c>
+      <c r="C356"/>
+      <c r="D356" t="s">
+        <v>230</v>
+      </c>
+      <c r="E356"/>
+      <c r="F356"/>
+      <c r="G356"/>
+      <c r="H356"/>
+      <c r="I356"/>
+      <c r="J356"/>
+      <c r="K356">
+        <v>6</v>
+      </c>
+      <c r="L356">
+        <v>4</v>
+      </c>
+      <c r="M356">
+        <v>24</v>
+      </c>
+      <c r="N356"/>
+    </row>
+    <row r="357" spans="1:14">
+      <c r="A357" t="s">
+        <v>376</v>
+      </c>
+      <c r="B357" t="s">
+        <v>377</v>
+      </c>
+      <c r="C357"/>
+      <c r="D357" t="s">
+        <v>28</v>
+      </c>
+      <c r="E357"/>
+      <c r="F357"/>
+      <c r="G357"/>
+      <c r="H357"/>
+      <c r="I357"/>
+      <c r="J357"/>
+      <c r="K357">
         <v>10</v>
       </c>
-      <c r="L352">
-        <v>4</v>
-      </c>
-      <c r="M352">
+      <c r="L357">
+        <v>1</v>
+      </c>
+      <c r="M357">
+        <v>10</v>
+      </c>
+      <c r="N357"/>
+    </row>
+    <row r="358" spans="1:14">
+      <c r="A358" t="s">
+        <v>378</v>
+      </c>
+      <c r="B358" t="s">
+        <v>379</v>
+      </c>
+      <c r="C358"/>
+      <c r="D358" t="s">
+        <v>20</v>
+      </c>
+      <c r="E358"/>
+      <c r="F358"/>
+      <c r="G358"/>
+      <c r="H358"/>
+      <c r="I358"/>
+      <c r="J358"/>
+      <c r="K358">
+        <v>10</v>
+      </c>
+      <c r="L358">
+        <v>4</v>
+      </c>
+      <c r="M358">
         <v>40</v>
       </c>
-      <c r="N352"/>
+      <c r="N358"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
Mise à jour Garde — 19/05/2026
</commit_message>
<xml_diff>
--- a/data/export_garde.xlsx
+++ b/data/export_garde.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="381">
   <si>
     <t>Début</t>
   </si>
@@ -1117,9 +1117,6 @@
     <t>16-05-2026</t>
   </si>
   <si>
-    <t>BSPP - Journée des CS</t>
-  </si>
-  <si>
     <t>CHTO</t>
   </si>
   <si>
@@ -1129,10 +1126,19 @@
     <t>23-05-2026</t>
   </si>
   <si>
+    <t>28-05-2026</t>
+  </si>
+  <si>
+    <t>[PROV] BSPP</t>
+  </si>
+  <si>
     <t>29-05-2026</t>
   </si>
   <si>
-    <t>[PROV] Garde BSPP</t>
+    <t xml:space="preserve"> Garde BSPP</t>
+  </si>
+  <si>
+    <t>02-06-2026</t>
   </si>
   <si>
     <t>06-06-2026</t>
@@ -1142,9 +1148,6 @@
   </si>
   <si>
     <t>09-06-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[PROV] Garde BSPP </t>
   </si>
   <si>
     <t>14-06-2026</t>
@@ -1513,7 +1516,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:N358"/>
+  <dimension ref="A1:N360"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854004" bestFit="true" customWidth="true" style="0"/>
@@ -13567,12 +13570,22 @@
       <c r="D346" t="s">
         <v>256</v>
       </c>
-      <c r="E346"/>
-      <c r="F346"/>
-      <c r="G346"/>
+      <c r="E346">
+        <v>0</v>
+      </c>
+      <c r="F346">
+        <v>0</v>
+      </c>
+      <c r="G346">
+        <v>0</v>
+      </c>
       <c r="H346"/>
-      <c r="I346"/>
-      <c r="J346"/>
+      <c r="I346">
+        <v>1</v>
+      </c>
+      <c r="J346">
+        <v>0</v>
+      </c>
       <c r="K346">
         <v>6</v>
       </c>
@@ -13595,12 +13608,24 @@
       <c r="D347" t="s">
         <v>256</v>
       </c>
-      <c r="E347"/>
-      <c r="F347"/>
-      <c r="G347"/>
-      <c r="H347"/>
-      <c r="I347"/>
-      <c r="J347"/>
+      <c r="E347">
+        <v>7</v>
+      </c>
+      <c r="F347">
+        <v>7</v>
+      </c>
+      <c r="G347">
+        <v>0</v>
+      </c>
+      <c r="H347">
+        <v>0</v>
+      </c>
+      <c r="I347">
+        <v>7</v>
+      </c>
+      <c r="J347">
+        <v>0</v>
+      </c>
       <c r="K347">
         <v>12</v>
       </c>
@@ -13617,26 +13642,38 @@
         <v>365</v>
       </c>
       <c r="B348" t="s">
-        <v>366</v>
+        <v>15</v>
       </c>
       <c r="C348"/>
       <c r="D348" t="s">
-        <v>367</v>
-      </c>
-      <c r="E348"/>
-      <c r="F348"/>
-      <c r="G348"/>
-      <c r="H348"/>
-      <c r="I348"/>
-      <c r="J348"/>
+        <v>366</v>
+      </c>
+      <c r="E348">
+        <v>6</v>
+      </c>
+      <c r="F348">
+        <v>5</v>
+      </c>
+      <c r="G348">
+        <v>0</v>
+      </c>
+      <c r="H348">
+        <v>0</v>
+      </c>
+      <c r="I348">
+        <v>5</v>
+      </c>
+      <c r="J348">
+        <v>0</v>
+      </c>
       <c r="K348">
         <v>8</v>
       </c>
       <c r="L348">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M348">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="N348"/>
     </row>
@@ -13661,16 +13698,16 @@
         <v>12</v>
       </c>
       <c r="L349">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M349">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="N349"/>
     </row>
     <row r="350" spans="1:14">
       <c r="A350" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B350" t="s">
         <v>227</v>
@@ -13698,7 +13735,7 @@
     </row>
     <row r="351" spans="1:14">
       <c r="A351" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B351" t="s">
         <v>227</v>
@@ -13717,23 +13754,23 @@
         <v>12</v>
       </c>
       <c r="L351">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M351">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="N351"/>
     </row>
     <row r="352" spans="1:14">
       <c r="A352" t="s">
+        <v>369</v>
+      </c>
+      <c r="B352" t="s">
         <v>370</v>
-      </c>
-      <c r="B352" t="s">
-        <v>371</v>
       </c>
       <c r="C352"/>
       <c r="D352" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="E352"/>
       <c r="F352"/>
@@ -13742,26 +13779,26 @@
       <c r="I352"/>
       <c r="J352"/>
       <c r="K352">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L352">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M352">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="N352"/>
     </row>
     <row r="353" spans="1:14">
       <c r="A353" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B353" t="s">
-        <v>371</v>
+        <v>227</v>
       </c>
       <c r="C353"/>
       <c r="D353" t="s">
-        <v>256</v>
+        <v>103</v>
       </c>
       <c r="E353"/>
       <c r="F353"/>
@@ -13770,26 +13807,26 @@
       <c r="I353"/>
       <c r="J353"/>
       <c r="K353">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="L353">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M353">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="N353"/>
     </row>
     <row r="354" spans="1:14">
       <c r="A354" t="s">
+        <v>371</v>
+      </c>
+      <c r="B354" t="s">
         <v>372</v>
-      </c>
-      <c r="B354" t="s">
-        <v>371</v>
       </c>
       <c r="C354"/>
       <c r="D354" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="E354"/>
       <c r="F354"/>
@@ -13798,13 +13835,13 @@
       <c r="I354"/>
       <c r="J354"/>
       <c r="K354">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L354">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M354">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="N354"/>
     </row>
@@ -13813,11 +13850,11 @@
         <v>373</v>
       </c>
       <c r="B355" t="s">
-        <v>371</v>
+        <v>15</v>
       </c>
       <c r="C355"/>
       <c r="D355" t="s">
-        <v>16</v>
+        <v>110</v>
       </c>
       <c r="E355"/>
       <c r="F355"/>
@@ -13829,10 +13866,10 @@
         <v>6</v>
       </c>
       <c r="L355">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M355">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="N355"/>
     </row>
@@ -13841,11 +13878,11 @@
         <v>374</v>
       </c>
       <c r="B356" t="s">
-        <v>375</v>
+        <v>227</v>
       </c>
       <c r="C356"/>
       <c r="D356" t="s">
-        <v>230</v>
+        <v>192</v>
       </c>
       <c r="E356"/>
       <c r="F356"/>
@@ -13854,26 +13891,26 @@
       <c r="I356"/>
       <c r="J356"/>
       <c r="K356">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="L356">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M356">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="N356"/>
     </row>
     <row r="357" spans="1:14">
       <c r="A357" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B357" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="C357"/>
       <c r="D357" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="E357"/>
       <c r="F357"/>
@@ -13882,26 +13919,26 @@
       <c r="I357"/>
       <c r="J357"/>
       <c r="K357">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L357">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M357">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="N357"/>
     </row>
     <row r="358" spans="1:14">
       <c r="A358" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B358" t="s">
-        <v>379</v>
+        <v>356</v>
       </c>
       <c r="C358"/>
       <c r="D358" t="s">
-        <v>20</v>
+        <v>230</v>
       </c>
       <c r="E358"/>
       <c r="F358"/>
@@ -13910,15 +13947,71 @@
       <c r="I358"/>
       <c r="J358"/>
       <c r="K358">
+        <v>6</v>
+      </c>
+      <c r="L358">
+        <v>5</v>
+      </c>
+      <c r="M358">
+        <v>30</v>
+      </c>
+      <c r="N358"/>
+    </row>
+    <row r="359" spans="1:14">
+      <c r="A359" t="s">
+        <v>377</v>
+      </c>
+      <c r="B359" t="s">
+        <v>378</v>
+      </c>
+      <c r="C359"/>
+      <c r="D359" t="s">
+        <v>28</v>
+      </c>
+      <c r="E359"/>
+      <c r="F359"/>
+      <c r="G359"/>
+      <c r="H359"/>
+      <c r="I359"/>
+      <c r="J359"/>
+      <c r="K359">
+        <v>9</v>
+      </c>
+      <c r="L359">
+        <v>3</v>
+      </c>
+      <c r="M359">
+        <v>27</v>
+      </c>
+      <c r="N359"/>
+    </row>
+    <row r="360" spans="1:14">
+      <c r="A360" t="s">
+        <v>379</v>
+      </c>
+      <c r="B360" t="s">
+        <v>380</v>
+      </c>
+      <c r="C360"/>
+      <c r="D360" t="s">
+        <v>20</v>
+      </c>
+      <c r="E360"/>
+      <c r="F360"/>
+      <c r="G360"/>
+      <c r="H360"/>
+      <c r="I360"/>
+      <c r="J360"/>
+      <c r="K360">
         <v>10</v>
       </c>
-      <c r="L358">
-        <v>4</v>
-      </c>
-      <c r="M358">
+      <c r="L360">
+        <v>4</v>
+      </c>
+      <c r="M360">
         <v>40</v>
       </c>
-      <c r="N358"/>
+      <c r="N360"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
Mise à jour Garde — 23/06/2026
</commit_message>
<xml_diff>
--- a/data/export_garde.xlsx
+++ b/data/export_garde.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="390">
   <si>
     <t>Début</t>
   </si>
@@ -1129,37 +1129,64 @@
     <t>28-05-2026</t>
   </si>
   <si>
+    <t>29-05-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Garde BSPP</t>
+  </si>
+  <si>
+    <t>02-06-2026</t>
+  </si>
+  <si>
+    <t>04-06-2026</t>
+  </si>
+  <si>
+    <t>06-06-2026</t>
+  </si>
+  <si>
+    <t>08-06-2026</t>
+  </si>
+  <si>
+    <t>09-06-2026</t>
+  </si>
+  <si>
+    <t>11-06-2026</t>
+  </si>
+  <si>
+    <t>14-06-2026</t>
+  </si>
+  <si>
+    <t>BSPP JPO CRET</t>
+  </si>
+  <si>
+    <t>19-06-2026</t>
+  </si>
+  <si>
+    <t>20-06-2026</t>
+  </si>
+  <si>
+    <t>BSPP JPO NATI</t>
+  </si>
+  <si>
+    <t>24-06-2026</t>
+  </si>
+  <si>
+    <t>30-06-2026</t>
+  </si>
+  <si>
+    <t>01-07-2026</t>
+  </si>
+  <si>
     <t>[PROV] BSPP</t>
   </si>
   <si>
-    <t>29-05-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Garde BSPP</t>
-  </si>
-  <si>
-    <t>02-06-2026</t>
-  </si>
-  <si>
-    <t>06-06-2026</t>
-  </si>
-  <si>
-    <t>08-06-2026</t>
-  </si>
-  <si>
-    <t>09-06-2026</t>
-  </si>
-  <si>
-    <t>14-06-2026</t>
-  </si>
-  <si>
-    <t>[PROV] BSPP JPO CRET</t>
-  </si>
-  <si>
-    <t>20-06-2026</t>
-  </si>
-  <si>
-    <t>[PROV] BSPP JPO NATI</t>
+    <t>07-07-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[PROV] BSPP </t>
+  </si>
+  <si>
+    <t>25-07-2026</t>
   </si>
 </sst>
 </file>
@@ -1516,7 +1543,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:N360"/>
+  <dimension ref="A1:N370"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854004" bestFit="true" customWidth="true" style="0"/>
@@ -13688,11 +13715,17 @@
       <c r="D349" t="s">
         <v>136</v>
       </c>
-      <c r="E349"/>
-      <c r="F349"/>
+      <c r="E349">
+        <v>4</v>
+      </c>
+      <c r="F349">
+        <v>2</v>
+      </c>
       <c r="G349"/>
       <c r="H349"/>
-      <c r="I349"/>
+      <c r="I349">
+        <v>3</v>
+      </c>
       <c r="J349"/>
       <c r="K349">
         <v>12</v>
@@ -13716,11 +13749,17 @@
       <c r="D350" t="s">
         <v>257</v>
       </c>
-      <c r="E350"/>
-      <c r="F350"/>
+      <c r="E350">
+        <v>3</v>
+      </c>
+      <c r="F350">
+        <v>3</v>
+      </c>
       <c r="G350"/>
       <c r="H350"/>
-      <c r="I350"/>
+      <c r="I350">
+        <v>3</v>
+      </c>
       <c r="J350"/>
       <c r="K350">
         <v>5</v>
@@ -13744,20 +13783,32 @@
       <c r="D351" t="s">
         <v>230</v>
       </c>
-      <c r="E351"/>
-      <c r="F351"/>
-      <c r="G351"/>
-      <c r="H351"/>
-      <c r="I351"/>
-      <c r="J351"/>
+      <c r="E351">
+        <v>7</v>
+      </c>
+      <c r="F351">
+        <v>7</v>
+      </c>
+      <c r="G351">
+        <v>0</v>
+      </c>
+      <c r="H351">
+        <v>0</v>
+      </c>
+      <c r="I351">
+        <v>7</v>
+      </c>
+      <c r="J351">
+        <v>0</v>
+      </c>
       <c r="K351">
         <v>12</v>
       </c>
       <c r="L351">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M351">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="N351"/>
     </row>
@@ -13766,32 +13817,44 @@
         <v>369</v>
       </c>
       <c r="B352" t="s">
-        <v>370</v>
+        <v>15</v>
       </c>
       <c r="C352"/>
       <c r="D352" t="s">
-        <v>93</v>
-      </c>
-      <c r="E352"/>
-      <c r="F352"/>
-      <c r="G352"/>
-      <c r="H352"/>
-      <c r="I352"/>
-      <c r="J352"/>
+        <v>256</v>
+      </c>
+      <c r="E352">
+        <v>3</v>
+      </c>
+      <c r="F352">
+        <v>2</v>
+      </c>
+      <c r="G352">
+        <v>0</v>
+      </c>
+      <c r="H352">
+        <v>0</v>
+      </c>
+      <c r="I352">
+        <v>2</v>
+      </c>
+      <c r="J352">
+        <v>0</v>
+      </c>
       <c r="K352">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="L352">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M352">
-        <v>6</v>
+        <v>16.5</v>
       </c>
       <c r="N352"/>
     </row>
     <row r="353" spans="1:14">
       <c r="A353" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B353" t="s">
         <v>227</v>
@@ -13800,12 +13863,22 @@
       <c r="D353" t="s">
         <v>103</v>
       </c>
-      <c r="E353"/>
-      <c r="F353"/>
-      <c r="G353"/>
+      <c r="E353">
+        <v>7</v>
+      </c>
+      <c r="F353">
+        <v>7</v>
+      </c>
+      <c r="G353">
+        <v>0</v>
+      </c>
       <c r="H353"/>
-      <c r="I353"/>
-      <c r="J353"/>
+      <c r="I353">
+        <v>8</v>
+      </c>
+      <c r="J353">
+        <v>0</v>
+      </c>
       <c r="K353">
         <v>12</v>
       </c>
@@ -13819,35 +13892,47 @@
     </row>
     <row r="354" spans="1:14">
       <c r="A354" t="s">
+        <v>370</v>
+      </c>
+      <c r="B354" t="s">
         <v>371</v>
-      </c>
-      <c r="B354" t="s">
-        <v>372</v>
       </c>
       <c r="C354"/>
       <c r="D354" t="s">
         <v>256</v>
       </c>
-      <c r="E354"/>
-      <c r="F354"/>
-      <c r="G354"/>
-      <c r="H354"/>
-      <c r="I354"/>
-      <c r="J354"/>
+      <c r="E354">
+        <v>6</v>
+      </c>
+      <c r="F354">
+        <v>4</v>
+      </c>
+      <c r="G354">
+        <v>0</v>
+      </c>
+      <c r="H354">
+        <v>0</v>
+      </c>
+      <c r="I354">
+        <v>6</v>
+      </c>
+      <c r="J354">
+        <v>0</v>
+      </c>
       <c r="K354">
         <v>6</v>
       </c>
       <c r="L354">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M354">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="N354"/>
     </row>
     <row r="355" spans="1:14">
       <c r="A355" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B355" t="s">
         <v>15</v>
@@ -13856,162 +13941,542 @@
       <c r="D355" t="s">
         <v>110</v>
       </c>
-      <c r="E355"/>
-      <c r="F355"/>
+      <c r="E355">
+        <v>4</v>
+      </c>
+      <c r="F355">
+        <v>4</v>
+      </c>
       <c r="G355"/>
       <c r="H355"/>
-      <c r="I355"/>
+      <c r="I355">
+        <v>4</v>
+      </c>
       <c r="J355"/>
       <c r="K355">
         <v>6</v>
       </c>
       <c r="L355">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M355">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="N355"/>
     </row>
     <row r="356" spans="1:14">
       <c r="A356" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B356" t="s">
-        <v>227</v>
+        <v>15</v>
       </c>
       <c r="C356"/>
       <c r="D356" t="s">
-        <v>192</v>
-      </c>
-      <c r="E356"/>
-      <c r="F356"/>
-      <c r="G356"/>
-      <c r="H356"/>
-      <c r="I356"/>
-      <c r="J356"/>
+        <v>167</v>
+      </c>
+      <c r="E356">
+        <v>4</v>
+      </c>
+      <c r="F356">
+        <v>3</v>
+      </c>
+      <c r="G356">
+        <v>0</v>
+      </c>
+      <c r="H356">
+        <v>0</v>
+      </c>
+      <c r="I356">
+        <v>4</v>
+      </c>
+      <c r="J356">
+        <v>0</v>
+      </c>
       <c r="K356">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L356">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M356">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="N356"/>
     </row>
     <row r="357" spans="1:14">
       <c r="A357" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B357" t="s">
-        <v>372</v>
+        <v>15</v>
       </c>
       <c r="C357"/>
       <c r="D357" t="s">
-        <v>16</v>
-      </c>
-      <c r="E357"/>
-      <c r="F357"/>
-      <c r="G357"/>
-      <c r="H357"/>
-      <c r="I357"/>
-      <c r="J357"/>
+        <v>366</v>
+      </c>
+      <c r="E357">
+        <v>4</v>
+      </c>
+      <c r="F357">
+        <v>4</v>
+      </c>
+      <c r="G357">
+        <v>0</v>
+      </c>
+      <c r="H357">
+        <v>0</v>
+      </c>
+      <c r="I357">
+        <v>4</v>
+      </c>
+      <c r="J357">
+        <v>0</v>
+      </c>
       <c r="K357">
         <v>6</v>
       </c>
       <c r="L357">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M357">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="N357"/>
     </row>
     <row r="358" spans="1:14">
       <c r="A358" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B358" t="s">
-        <v>356</v>
+        <v>227</v>
       </c>
       <c r="C358"/>
       <c r="D358" t="s">
-        <v>230</v>
-      </c>
-      <c r="E358"/>
-      <c r="F358"/>
-      <c r="G358"/>
+        <v>192</v>
+      </c>
+      <c r="E358">
+        <v>6</v>
+      </c>
+      <c r="F358">
+        <v>5</v>
+      </c>
+      <c r="G358">
+        <v>0</v>
+      </c>
       <c r="H358"/>
-      <c r="I358"/>
-      <c r="J358"/>
+      <c r="I358">
+        <v>6</v>
+      </c>
+      <c r="J358">
+        <v>0</v>
+      </c>
       <c r="K358">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="L358">
         <v>5</v>
       </c>
       <c r="M358">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="N358"/>
     </row>
     <row r="359" spans="1:14">
       <c r="A359" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B359" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="C359"/>
       <c r="D359" t="s">
-        <v>28</v>
-      </c>
-      <c r="E359"/>
-      <c r="F359"/>
-      <c r="G359"/>
+        <v>16</v>
+      </c>
+      <c r="E359">
+        <v>4</v>
+      </c>
+      <c r="F359">
+        <v>3</v>
+      </c>
+      <c r="G359">
+        <v>0</v>
+      </c>
       <c r="H359"/>
-      <c r="I359"/>
-      <c r="J359"/>
+      <c r="I359">
+        <v>4</v>
+      </c>
+      <c r="J359">
+        <v>0</v>
+      </c>
       <c r="K359">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L359">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M359">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="N359"/>
     </row>
     <row r="360" spans="1:14">
       <c r="A360" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="B360" t="s">
-        <v>380</v>
+        <v>356</v>
       </c>
       <c r="C360"/>
       <c r="D360" t="s">
+        <v>230</v>
+      </c>
+      <c r="E360">
+        <v>3</v>
+      </c>
+      <c r="F360">
+        <v>3</v>
+      </c>
+      <c r="G360">
+        <v>0</v>
+      </c>
+      <c r="H360"/>
+      <c r="I360">
+        <v>4</v>
+      </c>
+      <c r="J360">
+        <v>0</v>
+      </c>
+      <c r="K360">
+        <v>6</v>
+      </c>
+      <c r="L360">
+        <v>5</v>
+      </c>
+      <c r="M360">
+        <v>30</v>
+      </c>
+      <c r="N360"/>
+    </row>
+    <row r="361" spans="1:14">
+      <c r="A361" t="s">
+        <v>377</v>
+      </c>
+      <c r="B361" t="s">
+        <v>15</v>
+      </c>
+      <c r="C361"/>
+      <c r="D361" t="s">
+        <v>366</v>
+      </c>
+      <c r="E361">
+        <v>5</v>
+      </c>
+      <c r="F361">
+        <v>3</v>
+      </c>
+      <c r="G361">
+        <v>0</v>
+      </c>
+      <c r="H361">
+        <v>0</v>
+      </c>
+      <c r="I361">
+        <v>3</v>
+      </c>
+      <c r="J361">
+        <v>0</v>
+      </c>
+      <c r="K361">
+        <v>6</v>
+      </c>
+      <c r="L361">
+        <v>5</v>
+      </c>
+      <c r="M361">
+        <v>30</v>
+      </c>
+      <c r="N361"/>
+    </row>
+    <row r="362" spans="1:14">
+      <c r="A362" t="s">
+        <v>378</v>
+      </c>
+      <c r="B362" t="s">
+        <v>379</v>
+      </c>
+      <c r="C362"/>
+      <c r="D362" t="s">
+        <v>28</v>
+      </c>
+      <c r="E362">
+        <v>4</v>
+      </c>
+      <c r="F362">
+        <v>4</v>
+      </c>
+      <c r="G362"/>
+      <c r="H362"/>
+      <c r="I362">
+        <v>4</v>
+      </c>
+      <c r="J362"/>
+      <c r="K362">
+        <v>9</v>
+      </c>
+      <c r="L362">
+        <v>4</v>
+      </c>
+      <c r="M362">
+        <v>36</v>
+      </c>
+      <c r="N362"/>
+    </row>
+    <row r="363" spans="1:14">
+      <c r="A363" t="s">
+        <v>380</v>
+      </c>
+      <c r="B363" t="s">
+        <v>15</v>
+      </c>
+      <c r="C363"/>
+      <c r="D363" t="s">
+        <v>93</v>
+      </c>
+      <c r="E363">
+        <v>4</v>
+      </c>
+      <c r="F363">
+        <v>3</v>
+      </c>
+      <c r="G363">
+        <v>0</v>
+      </c>
+      <c r="H363">
+        <v>0</v>
+      </c>
+      <c r="I363">
+        <v>4</v>
+      </c>
+      <c r="J363">
+        <v>0</v>
+      </c>
+      <c r="K363">
+        <v>6</v>
+      </c>
+      <c r="L363">
+        <v>4</v>
+      </c>
+      <c r="M363">
+        <v>24</v>
+      </c>
+      <c r="N363"/>
+    </row>
+    <row r="364" spans="1:14">
+      <c r="A364" t="s">
+        <v>381</v>
+      </c>
+      <c r="B364" t="s">
+        <v>382</v>
+      </c>
+      <c r="C364"/>
+      <c r="D364" t="s">
         <v>20</v>
       </c>
-      <c r="E360"/>
-      <c r="F360"/>
-      <c r="G360"/>
-      <c r="H360"/>
-      <c r="I360"/>
-      <c r="J360"/>
-      <c r="K360">
+      <c r="E364">
+        <v>4</v>
+      </c>
+      <c r="F364">
+        <v>4</v>
+      </c>
+      <c r="G364">
+        <v>0</v>
+      </c>
+      <c r="H364">
+        <v>0</v>
+      </c>
+      <c r="I364">
+        <v>5</v>
+      </c>
+      <c r="J364">
+        <v>0</v>
+      </c>
+      <c r="K364">
         <v>10</v>
       </c>
-      <c r="L360">
-        <v>4</v>
-      </c>
-      <c r="M360">
+      <c r="L364">
+        <v>4</v>
+      </c>
+      <c r="M364">
         <v>40</v>
       </c>
-      <c r="N360"/>
+      <c r="N364"/>
+    </row>
+    <row r="365" spans="1:14">
+      <c r="A365" t="s">
+        <v>383</v>
+      </c>
+      <c r="B365" t="s">
+        <v>15</v>
+      </c>
+      <c r="C365"/>
+      <c r="D365" t="s">
+        <v>230</v>
+      </c>
+      <c r="E365"/>
+      <c r="F365"/>
+      <c r="G365"/>
+      <c r="H365"/>
+      <c r="I365"/>
+      <c r="J365"/>
+      <c r="K365">
+        <v>6</v>
+      </c>
+      <c r="L365">
+        <v>4</v>
+      </c>
+      <c r="M365">
+        <v>24</v>
+      </c>
+      <c r="N365"/>
+    </row>
+    <row r="366" spans="1:14">
+      <c r="A366" t="s">
+        <v>383</v>
+      </c>
+      <c r="B366" t="s">
+        <v>250</v>
+      </c>
+      <c r="C366"/>
+      <c r="D366"/>
+      <c r="E366"/>
+      <c r="F366"/>
+      <c r="G366"/>
+      <c r="H366"/>
+      <c r="I366"/>
+      <c r="J366"/>
+      <c r="K366">
+        <v>4.98</v>
+      </c>
+      <c r="L366">
+        <v>4</v>
+      </c>
+      <c r="M366">
+        <v>19.920000076294</v>
+      </c>
+      <c r="N366"/>
+    </row>
+    <row r="367" spans="1:14">
+      <c r="A367" t="s">
+        <v>384</v>
+      </c>
+      <c r="B367" t="s">
+        <v>15</v>
+      </c>
+      <c r="C367"/>
+      <c r="D367" t="s">
+        <v>256</v>
+      </c>
+      <c r="E367"/>
+      <c r="F367"/>
+      <c r="G367"/>
+      <c r="H367"/>
+      <c r="I367"/>
+      <c r="J367"/>
+      <c r="K367">
+        <v>6</v>
+      </c>
+      <c r="L367">
+        <v>4</v>
+      </c>
+      <c r="M367">
+        <v>24</v>
+      </c>
+      <c r="N367"/>
+    </row>
+    <row r="368" spans="1:14">
+      <c r="A368" t="s">
+        <v>385</v>
+      </c>
+      <c r="B368" t="s">
+        <v>386</v>
+      </c>
+      <c r="C368"/>
+      <c r="D368" t="s">
+        <v>366</v>
+      </c>
+      <c r="E368"/>
+      <c r="F368"/>
+      <c r="G368"/>
+      <c r="H368"/>
+      <c r="I368"/>
+      <c r="J368"/>
+      <c r="K368">
+        <v>6</v>
+      </c>
+      <c r="L368">
+        <v>4</v>
+      </c>
+      <c r="M368">
+        <v>24</v>
+      </c>
+      <c r="N368"/>
+    </row>
+    <row r="369" spans="1:14">
+      <c r="A369" t="s">
+        <v>387</v>
+      </c>
+      <c r="B369" t="s">
+        <v>388</v>
+      </c>
+      <c r="C369"/>
+      <c r="D369" t="s">
+        <v>161</v>
+      </c>
+      <c r="E369"/>
+      <c r="F369"/>
+      <c r="G369"/>
+      <c r="H369"/>
+      <c r="I369"/>
+      <c r="J369"/>
+      <c r="K369">
+        <v>6</v>
+      </c>
+      <c r="L369">
+        <v>1</v>
+      </c>
+      <c r="M369">
+        <v>6</v>
+      </c>
+      <c r="N369"/>
+    </row>
+    <row r="370" spans="1:14">
+      <c r="A370" t="s">
+        <v>389</v>
+      </c>
+      <c r="B370" t="s">
+        <v>15</v>
+      </c>
+      <c r="C370"/>
+      <c r="D370" t="s">
+        <v>256</v>
+      </c>
+      <c r="E370"/>
+      <c r="F370"/>
+      <c r="G370"/>
+      <c r="H370"/>
+      <c r="I370"/>
+      <c r="J370"/>
+      <c r="K370">
+        <v>12</v>
+      </c>
+      <c r="L370">
+        <v>3</v>
+      </c>
+      <c r="M370">
+        <v>36</v>
+      </c>
+      <c r="N370"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
Mise à jour Garde — 08/07/2026
</commit_message>
<xml_diff>
--- a/data/export_garde.xlsx
+++ b/data/export_garde.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="410">
   <si>
     <t>Début</t>
   </si>
@@ -1171,22 +1171,82 @@
     <t>24-06-2026</t>
   </si>
   <si>
+    <t>25-06-2026</t>
+  </si>
+  <si>
+    <t>26-06-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSPP canicule  </t>
+  </si>
+  <si>
+    <t>BITCH</t>
+  </si>
+  <si>
+    <t>27-06-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> bspp canicule </t>
+  </si>
+  <si>
+    <t>Boursault</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSPP canicule </t>
+  </si>
+  <si>
+    <t>28-06-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Garde BSPP canicule </t>
+  </si>
+  <si>
+    <t xml:space="preserve">garde canicule </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> garde canicule </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRET  </t>
+  </si>
+  <si>
     <t>30-06-2026</t>
   </si>
   <si>
     <t>01-07-2026</t>
   </si>
   <si>
+    <t>06-07-2026</t>
+  </si>
+  <si>
+    <t>07-07-2026</t>
+  </si>
+  <si>
+    <t>08-07-2026</t>
+  </si>
+  <si>
+    <t>12-07-2026</t>
+  </si>
+  <si>
     <t>[PROV] BSPP</t>
   </si>
   <si>
-    <t>07-07-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[PROV] BSPP </t>
-  </si>
-  <si>
-    <t>25-07-2026</t>
+    <t>13-07-2026</t>
+  </si>
+  <si>
+    <t>[pROV] BSPP</t>
+  </si>
+  <si>
+    <t>15-07-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHLY </t>
+  </si>
+  <si>
+    <t>21-07-2026</t>
+  </si>
+  <si>
+    <t>03-10-2026</t>
   </si>
 </sst>
 </file>
@@ -1543,7 +1603,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:N370"/>
+  <dimension ref="A1:N385"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854004" bestFit="true" customWidth="true" style="0"/>
@@ -14323,12 +14383,20 @@
       <c r="D365" t="s">
         <v>230</v>
       </c>
-      <c r="E365"/>
-      <c r="F365"/>
+      <c r="E365">
+        <v>5</v>
+      </c>
+      <c r="F365">
+        <v>3</v>
+      </c>
       <c r="G365"/>
       <c r="H365"/>
-      <c r="I365"/>
-      <c r="J365"/>
+      <c r="I365">
+        <v>5</v>
+      </c>
+      <c r="J365">
+        <v>1</v>
+      </c>
       <c r="K365">
         <v>6</v>
       </c>
@@ -14345,10 +14413,12 @@
         <v>383</v>
       </c>
       <c r="B366" t="s">
-        <v>250</v>
+        <v>36</v>
       </c>
       <c r="C366"/>
-      <c r="D366"/>
+      <c r="D366" t="s">
+        <v>37</v>
+      </c>
       <c r="E366"/>
       <c r="F366"/>
       <c r="G366"/>
@@ -14356,13 +14426,13 @@
       <c r="I366"/>
       <c r="J366"/>
       <c r="K366">
-        <v>4.98</v>
+        <v>5.98</v>
       </c>
       <c r="L366">
         <v>4</v>
       </c>
       <c r="M366">
-        <v>19.920000076294</v>
+        <v>23.920000076294</v>
       </c>
       <c r="N366"/>
     </row>
@@ -14375,108 +14445,622 @@
       </c>
       <c r="C367"/>
       <c r="D367" t="s">
-        <v>256</v>
+        <v>167</v>
       </c>
       <c r="E367"/>
-      <c r="F367"/>
+      <c r="F367">
+        <v>4</v>
+      </c>
       <c r="G367"/>
       <c r="H367"/>
-      <c r="I367"/>
+      <c r="I367">
+        <v>5</v>
+      </c>
       <c r="J367"/>
       <c r="K367">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L367">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M367">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="N367"/>
     </row>
     <row r="368" spans="1:14">
       <c r="A368" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B368" t="s">
-        <v>386</v>
+        <v>15</v>
       </c>
       <c r="C368"/>
       <c r="D368" t="s">
-        <v>366</v>
-      </c>
-      <c r="E368"/>
-      <c r="F368"/>
-      <c r="G368"/>
-      <c r="H368"/>
-      <c r="I368"/>
-      <c r="J368"/>
+        <v>110</v>
+      </c>
+      <c r="E368">
+        <v>3</v>
+      </c>
+      <c r="F368">
+        <v>2</v>
+      </c>
+      <c r="G368">
+        <v>0</v>
+      </c>
+      <c r="H368">
+        <v>0</v>
+      </c>
+      <c r="I368">
+        <v>3</v>
+      </c>
+      <c r="J368">
+        <v>0</v>
+      </c>
       <c r="K368">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L368">
         <v>4</v>
       </c>
       <c r="M368">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N368"/>
     </row>
     <row r="369" spans="1:14">
       <c r="A369" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B369" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C369"/>
       <c r="D369" t="s">
-        <v>161</v>
-      </c>
-      <c r="E369"/>
-      <c r="F369"/>
-      <c r="G369"/>
+        <v>387</v>
+      </c>
+      <c r="E369">
+        <v>7</v>
+      </c>
+      <c r="F369">
+        <v>6</v>
+      </c>
+      <c r="G369">
+        <v>0</v>
+      </c>
       <c r="H369"/>
-      <c r="I369"/>
-      <c r="J369"/>
+      <c r="I369">
+        <v>7</v>
+      </c>
+      <c r="J369">
+        <v>0</v>
+      </c>
       <c r="K369">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="L369">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M369">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="N369"/>
     </row>
     <row r="370" spans="1:14">
       <c r="A370" t="s">
+        <v>388</v>
+      </c>
+      <c r="B370" t="s">
         <v>389</v>
-      </c>
-      <c r="B370" t="s">
-        <v>15</v>
       </c>
       <c r="C370"/>
       <c r="D370" t="s">
-        <v>256</v>
-      </c>
-      <c r="E370"/>
-      <c r="F370"/>
+        <v>390</v>
+      </c>
+      <c r="E370">
+        <v>6</v>
+      </c>
+      <c r="F370">
+        <v>4</v>
+      </c>
       <c r="G370"/>
       <c r="H370"/>
-      <c r="I370"/>
-      <c r="J370"/>
+      <c r="I370">
+        <v>6</v>
+      </c>
+      <c r="J370">
+        <v>1</v>
+      </c>
       <c r="K370">
         <v>12</v>
       </c>
       <c r="L370">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M370">
+        <v>48</v>
+      </c>
+      <c r="N370"/>
+    </row>
+    <row r="371" spans="1:14">
+      <c r="A371" t="s">
+        <v>388</v>
+      </c>
+      <c r="B371" t="s">
+        <v>391</v>
+      </c>
+      <c r="C371"/>
+      <c r="D371" t="s">
+        <v>108</v>
+      </c>
+      <c r="E371">
+        <v>7</v>
+      </c>
+      <c r="F371">
+        <v>5</v>
+      </c>
+      <c r="G371">
+        <v>1</v>
+      </c>
+      <c r="H371">
+        <v>0</v>
+      </c>
+      <c r="I371">
+        <v>1</v>
+      </c>
+      <c r="J371">
+        <v>0</v>
+      </c>
+      <c r="K371">
+        <v>12</v>
+      </c>
+      <c r="L371">
+        <v>4</v>
+      </c>
+      <c r="M371">
+        <v>48</v>
+      </c>
+      <c r="N371"/>
+    </row>
+    <row r="372" spans="1:14">
+      <c r="A372" t="s">
+        <v>392</v>
+      </c>
+      <c r="B372" t="s">
+        <v>393</v>
+      </c>
+      <c r="C372"/>
+      <c r="D372" t="s">
+        <v>16</v>
+      </c>
+      <c r="E372">
+        <v>8</v>
+      </c>
+      <c r="F372">
+        <v>7</v>
+      </c>
+      <c r="G372">
+        <v>0</v>
+      </c>
+      <c r="H372"/>
+      <c r="I372">
+        <v>8</v>
+      </c>
+      <c r="J372">
+        <v>1</v>
+      </c>
+      <c r="K372">
+        <v>12</v>
+      </c>
+      <c r="L372">
+        <v>4</v>
+      </c>
+      <c r="M372">
+        <v>48</v>
+      </c>
+      <c r="N372"/>
+    </row>
+    <row r="373" spans="1:14">
+      <c r="A373" t="s">
+        <v>392</v>
+      </c>
+      <c r="B373" t="s">
+        <v>394</v>
+      </c>
+      <c r="C373"/>
+      <c r="D373" t="s">
+        <v>256</v>
+      </c>
+      <c r="E373"/>
+      <c r="F373"/>
+      <c r="G373"/>
+      <c r="H373"/>
+      <c r="I373"/>
+      <c r="J373"/>
+      <c r="K373">
+        <v>9.5</v>
+      </c>
+      <c r="L373">
+        <v>4</v>
+      </c>
+      <c r="M373">
+        <v>38</v>
+      </c>
+      <c r="N373"/>
+    </row>
+    <row r="374" spans="1:14">
+      <c r="A374" t="s">
+        <v>392</v>
+      </c>
+      <c r="B374" t="s">
+        <v>395</v>
+      </c>
+      <c r="C374"/>
+      <c r="D374" t="s">
+        <v>396</v>
+      </c>
+      <c r="E374"/>
+      <c r="F374"/>
+      <c r="G374"/>
+      <c r="H374"/>
+      <c r="I374"/>
+      <c r="J374"/>
+      <c r="K374">
+        <v>6</v>
+      </c>
+      <c r="L374">
+        <v>5</v>
+      </c>
+      <c r="M374">
+        <v>30</v>
+      </c>
+      <c r="N374"/>
+    </row>
+    <row r="375" spans="1:14">
+      <c r="A375" t="s">
+        <v>397</v>
+      </c>
+      <c r="B375" t="s">
+        <v>15</v>
+      </c>
+      <c r="C375"/>
+      <c r="D375" t="s">
+        <v>256</v>
+      </c>
+      <c r="E375">
+        <v>4</v>
+      </c>
+      <c r="F375">
+        <v>3</v>
+      </c>
+      <c r="G375"/>
+      <c r="H375"/>
+      <c r="I375">
+        <v>4</v>
+      </c>
+      <c r="J375">
+        <v>1</v>
+      </c>
+      <c r="K375">
+        <v>6</v>
+      </c>
+      <c r="L375">
+        <v>4</v>
+      </c>
+      <c r="M375">
+        <v>24</v>
+      </c>
+      <c r="N375"/>
+    </row>
+    <row r="376" spans="1:14">
+      <c r="A376" t="s">
+        <v>398</v>
+      </c>
+      <c r="B376" t="s">
+        <v>232</v>
+      </c>
+      <c r="C376"/>
+      <c r="D376" t="s">
+        <v>366</v>
+      </c>
+      <c r="E376">
+        <v>5</v>
+      </c>
+      <c r="F376">
+        <v>3</v>
+      </c>
+      <c r="G376"/>
+      <c r="H376"/>
+      <c r="I376">
+        <v>3</v>
+      </c>
+      <c r="J376"/>
+      <c r="K376">
+        <v>6</v>
+      </c>
+      <c r="L376">
+        <v>4</v>
+      </c>
+      <c r="M376">
+        <v>24</v>
+      </c>
+      <c r="N376"/>
+    </row>
+    <row r="377" spans="1:14">
+      <c r="A377" t="s">
+        <v>399</v>
+      </c>
+      <c r="B377" t="s">
+        <v>232</v>
+      </c>
+      <c r="C377"/>
+      <c r="D377" t="s">
+        <v>93</v>
+      </c>
+      <c r="E377">
+        <v>5</v>
+      </c>
+      <c r="F377">
+        <v>3</v>
+      </c>
+      <c r="G377">
+        <v>0</v>
+      </c>
+      <c r="H377">
+        <v>0</v>
+      </c>
+      <c r="I377">
+        <v>5</v>
+      </c>
+      <c r="J377">
+        <v>0</v>
+      </c>
+      <c r="K377">
+        <v>6</v>
+      </c>
+      <c r="L377">
+        <v>4</v>
+      </c>
+      <c r="M377">
+        <v>24</v>
+      </c>
+      <c r="N377"/>
+    </row>
+    <row r="378" spans="1:14">
+      <c r="A378" t="s">
+        <v>400</v>
+      </c>
+      <c r="B378" t="s">
+        <v>49</v>
+      </c>
+      <c r="C378"/>
+      <c r="D378" t="s">
+        <v>256</v>
+      </c>
+      <c r="E378">
+        <v>5</v>
+      </c>
+      <c r="F378">
+        <v>4</v>
+      </c>
+      <c r="G378">
+        <v>0</v>
+      </c>
+      <c r="H378">
+        <v>0</v>
+      </c>
+      <c r="I378">
+        <v>4</v>
+      </c>
+      <c r="J378">
+        <v>0</v>
+      </c>
+      <c r="K378">
+        <v>6</v>
+      </c>
+      <c r="L378">
+        <v>4</v>
+      </c>
+      <c r="M378">
+        <v>23</v>
+      </c>
+      <c r="N378"/>
+    </row>
+    <row r="379" spans="1:14">
+      <c r="A379" t="s">
+        <v>401</v>
+      </c>
+      <c r="B379" t="s">
+        <v>15</v>
+      </c>
+      <c r="C379"/>
+      <c r="D379" t="s">
+        <v>230</v>
+      </c>
+      <c r="E379"/>
+      <c r="F379"/>
+      <c r="G379"/>
+      <c r="H379"/>
+      <c r="I379"/>
+      <c r="J379"/>
+      <c r="K379">
+        <v>6</v>
+      </c>
+      <c r="L379">
+        <v>5</v>
+      </c>
+      <c r="M379">
+        <v>30</v>
+      </c>
+      <c r="N379"/>
+    </row>
+    <row r="380" spans="1:14">
+      <c r="A380" t="s">
+        <v>402</v>
+      </c>
+      <c r="B380" t="s">
+        <v>403</v>
+      </c>
+      <c r="C380"/>
+      <c r="D380" t="s">
+        <v>93</v>
+      </c>
+      <c r="E380"/>
+      <c r="F380"/>
+      <c r="G380"/>
+      <c r="H380"/>
+      <c r="I380"/>
+      <c r="J380"/>
+      <c r="K380">
+        <v>7</v>
+      </c>
+      <c r="L380">
+        <v>5</v>
+      </c>
+      <c r="M380">
+        <v>35</v>
+      </c>
+      <c r="N380"/>
+    </row>
+    <row r="381" spans="1:14">
+      <c r="A381" t="s">
+        <v>404</v>
+      </c>
+      <c r="B381" t="s">
+        <v>403</v>
+      </c>
+      <c r="C381"/>
+      <c r="D381" t="s">
+        <v>108</v>
+      </c>
+      <c r="E381"/>
+      <c r="F381"/>
+      <c r="G381"/>
+      <c r="H381"/>
+      <c r="I381"/>
+      <c r="J381"/>
+      <c r="K381">
+        <v>12</v>
+      </c>
+      <c r="L381">
+        <v>4</v>
+      </c>
+      <c r="M381">
+        <v>48</v>
+      </c>
+      <c r="N381"/>
+    </row>
+    <row r="382" spans="1:14">
+      <c r="A382" t="s">
+        <v>404</v>
+      </c>
+      <c r="B382" t="s">
+        <v>405</v>
+      </c>
+      <c r="C382"/>
+      <c r="D382" t="s">
+        <v>103</v>
+      </c>
+      <c r="E382"/>
+      <c r="F382"/>
+      <c r="G382"/>
+      <c r="H382"/>
+      <c r="I382"/>
+      <c r="J382"/>
+      <c r="K382">
+        <v>8</v>
+      </c>
+      <c r="L382">
+        <v>1</v>
+      </c>
+      <c r="M382">
+        <v>8</v>
+      </c>
+      <c r="N382"/>
+    </row>
+    <row r="383" spans="1:14">
+      <c r="A383" t="s">
+        <v>406</v>
+      </c>
+      <c r="B383" t="s">
+        <v>403</v>
+      </c>
+      <c r="C383"/>
+      <c r="D383" t="s">
+        <v>407</v>
+      </c>
+      <c r="E383"/>
+      <c r="F383"/>
+      <c r="G383"/>
+      <c r="H383"/>
+      <c r="I383"/>
+      <c r="J383"/>
+      <c r="K383">
+        <v>6</v>
+      </c>
+      <c r="L383">
+        <v>4</v>
+      </c>
+      <c r="M383">
+        <v>24</v>
+      </c>
+      <c r="N383"/>
+    </row>
+    <row r="384" spans="1:14">
+      <c r="A384" t="s">
+        <v>408</v>
+      </c>
+      <c r="B384" t="s">
+        <v>403</v>
+      </c>
+      <c r="C384"/>
+      <c r="D384" t="s">
+        <v>256</v>
+      </c>
+      <c r="E384"/>
+      <c r="F384"/>
+      <c r="G384"/>
+      <c r="H384"/>
+      <c r="I384"/>
+      <c r="J384"/>
+      <c r="K384">
+        <v>6</v>
+      </c>
+      <c r="L384">
+        <v>4</v>
+      </c>
+      <c r="M384">
+        <v>24</v>
+      </c>
+      <c r="N384"/>
+    </row>
+    <row r="385" spans="1:14">
+      <c r="A385" t="s">
+        <v>409</v>
+      </c>
+      <c r="B385" t="s">
+        <v>15</v>
+      </c>
+      <c r="C385"/>
+      <c r="D385" t="s">
+        <v>256</v>
+      </c>
+      <c r="E385"/>
+      <c r="F385"/>
+      <c r="G385"/>
+      <c r="H385"/>
+      <c r="I385"/>
+      <c r="J385"/>
+      <c r="K385">
+        <v>12</v>
+      </c>
+      <c r="L385">
+        <v>3</v>
+      </c>
+      <c r="M385">
         <v>36</v>
       </c>
-      <c r="N370"/>
+      <c r="N385"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>